<commit_message>
Prepare v1.3.0 release candidate
</commit_message>
<xml_diff>
--- a/examples/qualibact_ecoli/real_run_100/report/report.xlsx
+++ b/examples/qualibact_ecoli/real_run_100/report/report.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -753,7 +753,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -832,7 +832,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -907,7 +907,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -982,7 +982,7 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -1057,7 +1057,7 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -1136,7 +1136,7 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -1215,7 +1215,7 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -1294,7 +1294,7 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -1373,7 +1373,7 @@
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -1452,7 +1452,7 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -1531,7 +1531,7 @@
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -1610,7 +1610,7 @@
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -1689,7 +1689,7 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -1768,7 +1768,7 @@
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -1926,7 +1926,7 @@
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -2005,7 +2005,7 @@
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -2084,7 +2084,7 @@
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -2163,7 +2163,7 @@
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -2242,7 +2242,7 @@
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -2321,7 +2321,7 @@
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -2400,7 +2400,7 @@
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -2479,7 +2479,7 @@
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -2637,7 +2637,7 @@
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -2716,7 +2716,7 @@
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -2795,7 +2795,7 @@
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -2874,7 +2874,7 @@
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -2953,7 +2953,7 @@
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -3032,7 +3032,7 @@
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -3111,7 +3111,7 @@
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -3190,7 +3190,7 @@
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -3269,7 +3269,7 @@
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -3348,7 +3348,7 @@
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -3427,7 +3427,7 @@
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -3506,7 +3506,7 @@
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -3585,7 +3585,7 @@
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -3664,7 +3664,7 @@
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -3743,7 +3743,7 @@
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -3822,7 +3822,7 @@
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -3901,7 +3901,7 @@
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -3980,7 +3980,7 @@
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -4059,7 +4059,7 @@
       </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -4138,7 +4138,7 @@
       </c>
       <c r="S47" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -4217,7 +4217,7 @@
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -4296,7 +4296,7 @@
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -4375,7 +4375,7 @@
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -4454,7 +4454,7 @@
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -4533,7 +4533,7 @@
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -4612,7 +4612,7 @@
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -4691,7 +4691,7 @@
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -4770,7 +4770,7 @@
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -4849,7 +4849,7 @@
       </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -4928,7 +4928,7 @@
       </c>
       <c r="S57" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -5007,7 +5007,7 @@
       </c>
       <c r="S58" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -5086,7 +5086,7 @@
       </c>
       <c r="S59" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -5165,7 +5165,7 @@
       </c>
       <c r="S60" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -5244,7 +5244,7 @@
       </c>
       <c r="S61" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -5323,7 +5323,7 @@
       </c>
       <c r="S62" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -5402,7 +5402,7 @@
       </c>
       <c r="S63" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -5481,7 +5481,7 @@
       </c>
       <c r="S64" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -5560,7 +5560,7 @@
       </c>
       <c r="S65" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -5639,7 +5639,7 @@
       </c>
       <c r="S66" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -5718,7 +5718,7 @@
       </c>
       <c r="S67" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -5797,7 +5797,7 @@
       </c>
       <c r="S68" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -5876,7 +5876,7 @@
       </c>
       <c r="S69" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -5955,7 +5955,7 @@
       </c>
       <c r="S70" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -6034,7 +6034,7 @@
       </c>
       <c r="S71" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -6113,7 +6113,7 @@
       </c>
       <c r="S72" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -6192,7 +6192,7 @@
       </c>
       <c r="S73" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -6271,7 +6271,7 @@
       </c>
       <c r="S74" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -6350,7 +6350,7 @@
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -6429,7 +6429,7 @@
       </c>
       <c r="S76" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -6508,7 +6508,7 @@
       </c>
       <c r="S77" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -6587,7 +6587,7 @@
       </c>
       <c r="S78" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="S79" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -6745,7 +6745,7 @@
       </c>
       <c r="S80" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -6824,7 +6824,7 @@
       </c>
       <c r="S81" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -6903,7 +6903,7 @@
       </c>
       <c r="S82" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -6982,7 +6982,7 @@
       </c>
       <c r="S83" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -7061,7 +7061,7 @@
       </c>
       <c r="S84" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -7140,7 +7140,7 @@
       </c>
       <c r="S85" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -7219,7 +7219,7 @@
       </c>
       <c r="S86" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -7298,7 +7298,7 @@
       </c>
       <c r="S87" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -7377,7 +7377,7 @@
       </c>
       <c r="S88" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -7456,7 +7456,7 @@
       </c>
       <c r="S89" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -7535,7 +7535,7 @@
       </c>
       <c r="S90" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -7614,7 +7614,7 @@
       </c>
       <c r="S91" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -7693,7 +7693,7 @@
       </c>
       <c r="S92" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -7772,7 +7772,7 @@
       </c>
       <c r="S93" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -7851,7 +7851,7 @@
       </c>
       <c r="S94" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -7930,7 +7930,7 @@
       </c>
       <c r="S95" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -8009,7 +8009,7 @@
       </c>
       <c r="S96" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -8088,7 +8088,7 @@
       </c>
       <c r="S97" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -8167,7 +8167,7 @@
       </c>
       <c r="S98" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -8246,7 +8246,7 @@
       </c>
       <c r="S99" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -8325,7 +8325,7 @@
       </c>
       <c r="S100" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -8404,7 +8404,7 @@
       </c>
       <c r="S101" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -8594,7 +8594,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -8673,7 +8673,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -8752,7 +8752,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -8831,7 +8831,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -8906,7 +8906,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -8981,7 +8981,7 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -9056,7 +9056,7 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -9135,7 +9135,7 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -9214,7 +9214,7 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -9293,7 +9293,7 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -9372,7 +9372,7 @@
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -9451,7 +9451,7 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -9530,7 +9530,7 @@
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -9609,7 +9609,7 @@
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -9688,7 +9688,7 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -9767,7 +9767,7 @@
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -9846,7 +9846,7 @@
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -9925,7 +9925,7 @@
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -10004,7 +10004,7 @@
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -10083,7 +10083,7 @@
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -10162,7 +10162,7 @@
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -10241,7 +10241,7 @@
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -10320,7 +10320,7 @@
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -10399,7 +10399,7 @@
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -10478,7 +10478,7 @@
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -10557,7 +10557,7 @@
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -10636,7 +10636,7 @@
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -10715,7 +10715,7 @@
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -10794,7 +10794,7 @@
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -10873,7 +10873,7 @@
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -10952,7 +10952,7 @@
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -11031,7 +11031,7 @@
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -11110,7 +11110,7 @@
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -11189,7 +11189,7 @@
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -11268,7 +11268,7 @@
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -11347,7 +11347,7 @@
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -11426,7 +11426,7 @@
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -11505,7 +11505,7 @@
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -11584,7 +11584,7 @@
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -11663,7 +11663,7 @@
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -11742,7 +11742,7 @@
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -11821,7 +11821,7 @@
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -11900,7 +11900,7 @@
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -11979,7 +11979,7 @@
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -12058,7 +12058,7 @@
       </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -12137,7 +12137,7 @@
       </c>
       <c r="S47" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -12216,7 +12216,7 @@
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -12295,7 +12295,7 @@
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -12374,7 +12374,7 @@
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -12453,7 +12453,7 @@
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -12532,7 +12532,7 @@
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -12611,7 +12611,7 @@
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -12690,7 +12690,7 @@
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -12769,7 +12769,7 @@
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -12848,7 +12848,7 @@
       </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -12927,7 +12927,7 @@
       </c>
       <c r="S57" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -13006,7 +13006,7 @@
       </c>
       <c r="S58" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -13085,7 +13085,7 @@
       </c>
       <c r="S59" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -13164,7 +13164,7 @@
       </c>
       <c r="S60" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -13243,7 +13243,7 @@
       </c>
       <c r="S61" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -13322,7 +13322,7 @@
       </c>
       <c r="S62" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -13401,7 +13401,7 @@
       </c>
       <c r="S63" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -13480,7 +13480,7 @@
       </c>
       <c r="S64" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -13559,7 +13559,7 @@
       </c>
       <c r="S65" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -13638,7 +13638,7 @@
       </c>
       <c r="S66" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -13717,7 +13717,7 @@
       </c>
       <c r="S67" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -13796,7 +13796,7 @@
       </c>
       <c r="S68" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -13875,7 +13875,7 @@
       </c>
       <c r="S69" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -13954,7 +13954,7 @@
       </c>
       <c r="S70" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -14033,7 +14033,7 @@
       </c>
       <c r="S71" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -14112,7 +14112,7 @@
       </c>
       <c r="S72" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -14191,7 +14191,7 @@
       </c>
       <c r="S73" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -14270,7 +14270,7 @@
       </c>
       <c r="S74" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -14349,7 +14349,7 @@
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -14428,7 +14428,7 @@
       </c>
       <c r="S76" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -14507,7 +14507,7 @@
       </c>
       <c r="S77" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -14586,7 +14586,7 @@
       </c>
       <c r="S78" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -14665,7 +14665,7 @@
       </c>
       <c r="S79" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -14744,7 +14744,7 @@
       </c>
       <c r="S80" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -14823,7 +14823,7 @@
       </c>
       <c r="S81" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -14902,7 +14902,7 @@
       </c>
       <c r="S82" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -14981,7 +14981,7 @@
       </c>
       <c r="S83" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -15060,7 +15060,7 @@
       </c>
       <c r="S84" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -15139,7 +15139,7 @@
       </c>
       <c r="S85" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -15218,7 +15218,7 @@
       </c>
       <c r="S86" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -15297,7 +15297,7 @@
       </c>
       <c r="S87" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -15376,7 +15376,7 @@
       </c>
       <c r="S88" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -15455,7 +15455,7 @@
       </c>
       <c r="S89" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -15534,7 +15534,7 @@
       </c>
       <c r="S90" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -15613,7 +15613,7 @@
       </c>
       <c r="S91" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -15692,7 +15692,7 @@
       </c>
       <c r="S92" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -15771,7 +15771,7 @@
       </c>
       <c r="S93" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -15850,7 +15850,7 @@
       </c>
       <c r="S94" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -15929,7 +15929,7 @@
       </c>
       <c r="S95" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -16008,7 +16008,7 @@
       </c>
       <c r="S96" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -16087,7 +16087,7 @@
       </c>
       <c r="S97" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -16166,7 +16166,7 @@
       </c>
       <c r="S98" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -16245,7 +16245,7 @@
       </c>
       <c r="S99" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -16324,7 +16324,7 @@
       </c>
       <c r="S100" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -16403,7 +16403,7 @@
       </c>
       <c r="S101" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
     </row>
@@ -17144,17 +17144,17 @@
       </c>
       <c r="BU2" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV2" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW2" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX2" t="inlineStr">
@@ -17202,7 +17202,7 @@
       </c>
       <c r="CG2" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH2" t="inlineStr">
@@ -17502,17 +17502,17 @@
       </c>
       <c r="BU3" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV3" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW3" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX3" t="inlineStr">
@@ -17560,7 +17560,7 @@
       </c>
       <c r="CG3" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH3" t="inlineStr">
@@ -17860,17 +17860,17 @@
       </c>
       <c r="BU4" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV4" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW4" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX4" t="inlineStr">
@@ -17918,7 +17918,7 @@
       </c>
       <c r="CG4" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH4" t="inlineStr">
@@ -18218,17 +18218,17 @@
       </c>
       <c r="BU5" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV5" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW5" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX5" t="inlineStr">
@@ -18276,7 +18276,7 @@
       </c>
       <c r="CG5" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH5" t="inlineStr">
@@ -18572,17 +18572,17 @@
       </c>
       <c r="BU6" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV6" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW6" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX6" t="inlineStr">
@@ -18626,7 +18626,7 @@
       <c r="CF6" t="inlineStr"/>
       <c r="CG6" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH6" t="inlineStr">
@@ -18922,17 +18922,17 @@
       </c>
       <c r="BU7" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV7" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW7" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX7" t="inlineStr">
@@ -18976,7 +18976,7 @@
       <c r="CF7" t="inlineStr"/>
       <c r="CG7" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH7" t="inlineStr">
@@ -19272,17 +19272,17 @@
       </c>
       <c r="BU8" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV8" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW8" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX8" t="inlineStr">
@@ -19326,7 +19326,7 @@
       <c r="CF8" t="inlineStr"/>
       <c r="CG8" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH8" t="inlineStr">
@@ -19626,17 +19626,17 @@
       </c>
       <c r="BU9" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV9" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW9" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX9" t="inlineStr">
@@ -19684,7 +19684,7 @@
       </c>
       <c r="CG9" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH9" t="inlineStr">
@@ -19984,17 +19984,17 @@
       </c>
       <c r="BU10" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV10" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW10" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX10" t="inlineStr">
@@ -20042,7 +20042,7 @@
       </c>
       <c r="CG10" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH10" t="inlineStr">
@@ -20342,17 +20342,17 @@
       </c>
       <c r="BU11" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV11" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW11" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX11" t="inlineStr">
@@ -20400,7 +20400,7 @@
       </c>
       <c r="CG11" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH11" t="inlineStr">
@@ -20700,17 +20700,17 @@
       </c>
       <c r="BU12" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV12" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW12" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX12" t="inlineStr">
@@ -20758,7 +20758,7 @@
       </c>
       <c r="CG12" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH12" t="inlineStr">
@@ -21058,17 +21058,17 @@
       </c>
       <c r="BU13" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV13" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW13" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX13" t="inlineStr">
@@ -21116,7 +21116,7 @@
       </c>
       <c r="CG13" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH13" t="inlineStr">
@@ -21416,17 +21416,17 @@
       </c>
       <c r="BU14" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV14" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW14" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX14" t="inlineStr">
@@ -21474,7 +21474,7 @@
       </c>
       <c r="CG14" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH14" t="inlineStr">
@@ -21774,17 +21774,17 @@
       </c>
       <c r="BU15" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV15" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW15" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX15" t="inlineStr">
@@ -21832,7 +21832,7 @@
       </c>
       <c r="CG15" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH15" t="inlineStr">
@@ -22132,17 +22132,17 @@
       </c>
       <c r="BU16" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV16" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW16" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX16" t="inlineStr">
@@ -22190,7 +22190,7 @@
       </c>
       <c r="CG16" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH16" t="inlineStr">
@@ -22490,17 +22490,17 @@
       </c>
       <c r="BU17" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV17" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW17" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX17" t="inlineStr">
@@ -22548,7 +22548,7 @@
       </c>
       <c r="CG17" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH17" t="inlineStr">
@@ -22848,17 +22848,17 @@
       </c>
       <c r="BU18" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV18" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW18" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX18" t="inlineStr">
@@ -22906,7 +22906,7 @@
       </c>
       <c r="CG18" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH18" t="inlineStr">
@@ -23206,17 +23206,17 @@
       </c>
       <c r="BU19" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV19" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW19" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX19" t="inlineStr">
@@ -23264,7 +23264,7 @@
       </c>
       <c r="CG19" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH19" t="inlineStr">
@@ -23564,17 +23564,17 @@
       </c>
       <c r="BU20" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV20" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW20" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX20" t="inlineStr">
@@ -23622,7 +23622,7 @@
       </c>
       <c r="CG20" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH20" t="inlineStr">
@@ -23922,17 +23922,17 @@
       </c>
       <c r="BU21" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV21" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW21" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX21" t="inlineStr">
@@ -23980,7 +23980,7 @@
       </c>
       <c r="CG21" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH21" t="inlineStr">
@@ -24280,17 +24280,17 @@
       </c>
       <c r="BU22" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV22" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW22" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX22" t="inlineStr">
@@ -24338,7 +24338,7 @@
       </c>
       <c r="CG22" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH22" t="inlineStr">
@@ -24638,17 +24638,17 @@
       </c>
       <c r="BU23" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV23" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW23" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX23" t="inlineStr">
@@ -24696,7 +24696,7 @@
       </c>
       <c r="CG23" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH23" t="inlineStr">
@@ -24996,17 +24996,17 @@
       </c>
       <c r="BU24" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV24" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW24" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX24" t="inlineStr">
@@ -25054,7 +25054,7 @@
       </c>
       <c r="CG24" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH24" t="inlineStr">
@@ -25354,17 +25354,17 @@
       </c>
       <c r="BU25" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV25" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW25" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX25" t="inlineStr">
@@ -25412,7 +25412,7 @@
       </c>
       <c r="CG25" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH25" t="inlineStr">
@@ -25712,17 +25712,17 @@
       </c>
       <c r="BU26" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV26" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW26" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX26" t="inlineStr">
@@ -25770,7 +25770,7 @@
       </c>
       <c r="CG26" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH26" t="inlineStr">
@@ -26070,17 +26070,17 @@
       </c>
       <c r="BU27" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV27" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW27" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX27" t="inlineStr">
@@ -26128,7 +26128,7 @@
       </c>
       <c r="CG27" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH27" t="inlineStr">
@@ -26428,17 +26428,17 @@
       </c>
       <c r="BU28" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV28" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW28" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX28" t="inlineStr">
@@ -26486,7 +26486,7 @@
       </c>
       <c r="CG28" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH28" t="inlineStr">
@@ -26786,17 +26786,17 @@
       </c>
       <c r="BU29" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV29" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW29" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX29" t="inlineStr">
@@ -26844,7 +26844,7 @@
       </c>
       <c r="CG29" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH29" t="inlineStr">
@@ -27144,17 +27144,17 @@
       </c>
       <c r="BU30" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV30" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW30" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX30" t="inlineStr">
@@ -27202,7 +27202,7 @@
       </c>
       <c r="CG30" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH30" t="inlineStr">
@@ -27502,17 +27502,17 @@
       </c>
       <c r="BU31" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV31" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW31" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX31" t="inlineStr">
@@ -27560,7 +27560,7 @@
       </c>
       <c r="CG31" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH31" t="inlineStr">
@@ -27860,17 +27860,17 @@
       </c>
       <c r="BU32" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV32" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW32" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX32" t="inlineStr">
@@ -27918,7 +27918,7 @@
       </c>
       <c r="CG32" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH32" t="inlineStr">
@@ -28218,17 +28218,17 @@
       </c>
       <c r="BU33" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV33" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW33" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX33" t="inlineStr">
@@ -28276,7 +28276,7 @@
       </c>
       <c r="CG33" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH33" t="inlineStr">
@@ -28576,17 +28576,17 @@
       </c>
       <c r="BU34" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV34" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW34" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX34" t="inlineStr">
@@ -28634,7 +28634,7 @@
       </c>
       <c r="CG34" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH34" t="inlineStr">
@@ -28934,17 +28934,17 @@
       </c>
       <c r="BU35" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV35" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW35" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX35" t="inlineStr">
@@ -28992,7 +28992,7 @@
       </c>
       <c r="CG35" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH35" t="inlineStr">
@@ -29292,17 +29292,17 @@
       </c>
       <c r="BU36" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV36" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW36" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX36" t="inlineStr">
@@ -29350,7 +29350,7 @@
       </c>
       <c r="CG36" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH36" t="inlineStr">
@@ -29650,17 +29650,17 @@
       </c>
       <c r="BU37" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV37" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW37" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX37" t="inlineStr">
@@ -29708,7 +29708,7 @@
       </c>
       <c r="CG37" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH37" t="inlineStr">
@@ -30008,17 +30008,17 @@
       </c>
       <c r="BU38" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV38" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW38" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX38" t="inlineStr">
@@ -30066,7 +30066,7 @@
       </c>
       <c r="CG38" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH38" t="inlineStr">
@@ -30366,17 +30366,17 @@
       </c>
       <c r="BU39" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV39" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW39" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX39" t="inlineStr">
@@ -30424,7 +30424,7 @@
       </c>
       <c r="CG39" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH39" t="inlineStr">
@@ -30724,17 +30724,17 @@
       </c>
       <c r="BU40" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV40" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW40" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX40" t="inlineStr">
@@ -30782,7 +30782,7 @@
       </c>
       <c r="CG40" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH40" t="inlineStr">
@@ -31082,17 +31082,17 @@
       </c>
       <c r="BU41" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV41" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW41" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX41" t="inlineStr">
@@ -31140,7 +31140,7 @@
       </c>
       <c r="CG41" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH41" t="inlineStr">
@@ -31440,17 +31440,17 @@
       </c>
       <c r="BU42" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV42" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW42" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX42" t="inlineStr">
@@ -31498,7 +31498,7 @@
       </c>
       <c r="CG42" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH42" t="inlineStr">
@@ -31798,17 +31798,17 @@
       </c>
       <c r="BU43" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV43" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW43" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX43" t="inlineStr">
@@ -31856,7 +31856,7 @@
       </c>
       <c r="CG43" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH43" t="inlineStr">
@@ -32156,17 +32156,17 @@
       </c>
       <c r="BU44" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV44" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW44" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX44" t="inlineStr">
@@ -32214,7 +32214,7 @@
       </c>
       <c r="CG44" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH44" t="inlineStr">
@@ -32514,17 +32514,17 @@
       </c>
       <c r="BU45" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV45" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW45" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX45" t="inlineStr">
@@ -32572,7 +32572,7 @@
       </c>
       <c r="CG45" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH45" t="inlineStr">
@@ -32872,17 +32872,17 @@
       </c>
       <c r="BU46" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV46" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW46" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX46" t="inlineStr">
@@ -32930,7 +32930,7 @@
       </c>
       <c r="CG46" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH46" t="inlineStr">
@@ -33230,17 +33230,17 @@
       </c>
       <c r="BU47" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV47" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW47" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX47" t="inlineStr">
@@ -33288,7 +33288,7 @@
       </c>
       <c r="CG47" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH47" t="inlineStr">
@@ -33588,17 +33588,17 @@
       </c>
       <c r="BU48" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV48" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW48" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX48" t="inlineStr">
@@ -33646,7 +33646,7 @@
       </c>
       <c r="CG48" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH48" t="inlineStr">
@@ -33946,17 +33946,17 @@
       </c>
       <c r="BU49" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV49" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW49" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX49" t="inlineStr">
@@ -34004,7 +34004,7 @@
       </c>
       <c r="CG49" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH49" t="inlineStr">
@@ -34304,17 +34304,17 @@
       </c>
       <c r="BU50" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV50" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW50" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX50" t="inlineStr">
@@ -34362,7 +34362,7 @@
       </c>
       <c r="CG50" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH50" t="inlineStr">
@@ -34662,17 +34662,17 @@
       </c>
       <c r="BU51" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV51" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW51" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX51" t="inlineStr">
@@ -34720,7 +34720,7 @@
       </c>
       <c r="CG51" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH51" t="inlineStr">
@@ -35020,17 +35020,17 @@
       </c>
       <c r="BU52" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV52" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW52" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX52" t="inlineStr">
@@ -35078,7 +35078,7 @@
       </c>
       <c r="CG52" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH52" t="inlineStr">
@@ -35378,17 +35378,17 @@
       </c>
       <c r="BU53" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV53" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW53" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX53" t="inlineStr">
@@ -35436,7 +35436,7 @@
       </c>
       <c r="CG53" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH53" t="inlineStr">
@@ -35736,17 +35736,17 @@
       </c>
       <c r="BU54" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV54" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW54" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX54" t="inlineStr">
@@ -35794,7 +35794,7 @@
       </c>
       <c r="CG54" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH54" t="inlineStr">
@@ -36094,17 +36094,17 @@
       </c>
       <c r="BU55" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV55" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW55" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX55" t="inlineStr">
@@ -36152,7 +36152,7 @@
       </c>
       <c r="CG55" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH55" t="inlineStr">
@@ -36452,17 +36452,17 @@
       </c>
       <c r="BU56" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV56" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW56" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX56" t="inlineStr">
@@ -36510,7 +36510,7 @@
       </c>
       <c r="CG56" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH56" t="inlineStr">
@@ -36810,17 +36810,17 @@
       </c>
       <c r="BU57" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV57" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW57" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX57" t="inlineStr">
@@ -36868,7 +36868,7 @@
       </c>
       <c r="CG57" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH57" t="inlineStr">
@@ -37168,17 +37168,17 @@
       </c>
       <c r="BU58" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV58" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW58" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX58" t="inlineStr">
@@ -37226,7 +37226,7 @@
       </c>
       <c r="CG58" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH58" t="inlineStr">
@@ -37526,17 +37526,17 @@
       </c>
       <c r="BU59" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV59" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW59" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX59" t="inlineStr">
@@ -37584,7 +37584,7 @@
       </c>
       <c r="CG59" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH59" t="inlineStr">
@@ -37884,17 +37884,17 @@
       </c>
       <c r="BU60" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV60" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW60" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX60" t="inlineStr">
@@ -37942,7 +37942,7 @@
       </c>
       <c r="CG60" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH60" t="inlineStr">
@@ -38242,17 +38242,17 @@
       </c>
       <c r="BU61" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV61" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW61" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX61" t="inlineStr">
@@ -38300,7 +38300,7 @@
       </c>
       <c r="CG61" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH61" t="inlineStr">
@@ -38600,17 +38600,17 @@
       </c>
       <c r="BU62" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV62" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW62" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX62" t="inlineStr">
@@ -38658,7 +38658,7 @@
       </c>
       <c r="CG62" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH62" t="inlineStr">
@@ -38958,17 +38958,17 @@
       </c>
       <c r="BU63" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV63" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW63" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX63" t="inlineStr">
@@ -39016,7 +39016,7 @@
       </c>
       <c r="CG63" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH63" t="inlineStr">
@@ -39316,17 +39316,17 @@
       </c>
       <c r="BU64" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV64" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW64" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX64" t="inlineStr">
@@ -39374,7 +39374,7 @@
       </c>
       <c r="CG64" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH64" t="inlineStr">
@@ -39674,17 +39674,17 @@
       </c>
       <c r="BU65" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV65" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW65" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX65" t="inlineStr">
@@ -39732,7 +39732,7 @@
       </c>
       <c r="CG65" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH65" t="inlineStr">
@@ -40032,17 +40032,17 @@
       </c>
       <c r="BU66" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV66" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW66" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX66" t="inlineStr">
@@ -40090,7 +40090,7 @@
       </c>
       <c r="CG66" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH66" t="inlineStr">
@@ -40390,17 +40390,17 @@
       </c>
       <c r="BU67" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV67" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW67" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX67" t="inlineStr">
@@ -40448,7 +40448,7 @@
       </c>
       <c r="CG67" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH67" t="inlineStr">
@@ -40748,17 +40748,17 @@
       </c>
       <c r="BU68" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV68" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW68" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX68" t="inlineStr">
@@ -40806,7 +40806,7 @@
       </c>
       <c r="CG68" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH68" t="inlineStr">
@@ -41106,17 +41106,17 @@
       </c>
       <c r="BU69" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV69" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW69" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX69" t="inlineStr">
@@ -41164,7 +41164,7 @@
       </c>
       <c r="CG69" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH69" t="inlineStr">
@@ -41464,17 +41464,17 @@
       </c>
       <c r="BU70" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV70" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW70" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX70" t="inlineStr">
@@ -41522,7 +41522,7 @@
       </c>
       <c r="CG70" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH70" t="inlineStr">
@@ -41822,17 +41822,17 @@
       </c>
       <c r="BU71" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV71" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW71" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX71" t="inlineStr">
@@ -41880,7 +41880,7 @@
       </c>
       <c r="CG71" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH71" t="inlineStr">
@@ -42180,17 +42180,17 @@
       </c>
       <c r="BU72" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV72" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW72" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX72" t="inlineStr">
@@ -42238,7 +42238,7 @@
       </c>
       <c r="CG72" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH72" t="inlineStr">
@@ -42538,17 +42538,17 @@
       </c>
       <c r="BU73" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV73" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW73" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX73" t="inlineStr">
@@ -42596,7 +42596,7 @@
       </c>
       <c r="CG73" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH73" t="inlineStr">
@@ -42896,17 +42896,17 @@
       </c>
       <c r="BU74" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV74" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW74" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX74" t="inlineStr">
@@ -42954,7 +42954,7 @@
       </c>
       <c r="CG74" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH74" t="inlineStr">
@@ -43254,17 +43254,17 @@
       </c>
       <c r="BU75" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV75" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW75" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX75" t="inlineStr">
@@ -43312,7 +43312,7 @@
       </c>
       <c r="CG75" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH75" t="inlineStr">
@@ -43612,17 +43612,17 @@
       </c>
       <c r="BU76" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV76" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW76" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX76" t="inlineStr">
@@ -43670,7 +43670,7 @@
       </c>
       <c r="CG76" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH76" t="inlineStr">
@@ -43970,17 +43970,17 @@
       </c>
       <c r="BU77" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV77" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW77" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX77" t="inlineStr">
@@ -44028,7 +44028,7 @@
       </c>
       <c r="CG77" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH77" t="inlineStr">
@@ -44328,17 +44328,17 @@
       </c>
       <c r="BU78" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV78" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW78" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX78" t="inlineStr">
@@ -44386,7 +44386,7 @@
       </c>
       <c r="CG78" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH78" t="inlineStr">
@@ -44686,17 +44686,17 @@
       </c>
       <c r="BU79" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV79" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW79" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX79" t="inlineStr">
@@ -44744,7 +44744,7 @@
       </c>
       <c r="CG79" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH79" t="inlineStr">
@@ -45044,17 +45044,17 @@
       </c>
       <c r="BU80" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV80" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW80" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX80" t="inlineStr">
@@ -45102,7 +45102,7 @@
       </c>
       <c r="CG80" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH80" t="inlineStr">
@@ -45402,17 +45402,17 @@
       </c>
       <c r="BU81" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV81" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW81" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX81" t="inlineStr">
@@ -45460,7 +45460,7 @@
       </c>
       <c r="CG81" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH81" t="inlineStr">
@@ -45760,17 +45760,17 @@
       </c>
       <c r="BU82" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV82" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW82" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX82" t="inlineStr">
@@ -45818,7 +45818,7 @@
       </c>
       <c r="CG82" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH82" t="inlineStr">
@@ -46118,17 +46118,17 @@
       </c>
       <c r="BU83" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV83" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW83" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX83" t="inlineStr">
@@ -46176,7 +46176,7 @@
       </c>
       <c r="CG83" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH83" t="inlineStr">
@@ -46476,17 +46476,17 @@
       </c>
       <c r="BU84" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV84" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW84" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX84" t="inlineStr">
@@ -46534,7 +46534,7 @@
       </c>
       <c r="CG84" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH84" t="inlineStr">
@@ -46834,17 +46834,17 @@
       </c>
       <c r="BU85" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV85" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW85" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX85" t="inlineStr">
@@ -46892,7 +46892,7 @@
       </c>
       <c r="CG85" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH85" t="inlineStr">
@@ -47192,17 +47192,17 @@
       </c>
       <c r="BU86" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV86" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW86" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX86" t="inlineStr">
@@ -47250,7 +47250,7 @@
       </c>
       <c r="CG86" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH86" t="inlineStr">
@@ -47550,17 +47550,17 @@
       </c>
       <c r="BU87" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV87" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW87" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX87" t="inlineStr">
@@ -47608,7 +47608,7 @@
       </c>
       <c r="CG87" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH87" t="inlineStr">
@@ -47908,17 +47908,17 @@
       </c>
       <c r="BU88" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV88" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW88" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX88" t="inlineStr">
@@ -47966,7 +47966,7 @@
       </c>
       <c r="CG88" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH88" t="inlineStr">
@@ -48266,17 +48266,17 @@
       </c>
       <c r="BU89" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV89" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW89" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX89" t="inlineStr">
@@ -48324,7 +48324,7 @@
       </c>
       <c r="CG89" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH89" t="inlineStr">
@@ -48624,17 +48624,17 @@
       </c>
       <c r="BU90" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV90" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW90" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX90" t="inlineStr">
@@ -48682,7 +48682,7 @@
       </c>
       <c r="CG90" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH90" t="inlineStr">
@@ -48982,17 +48982,17 @@
       </c>
       <c r="BU91" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV91" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW91" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX91" t="inlineStr">
@@ -49040,7 +49040,7 @@
       </c>
       <c r="CG91" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH91" t="inlineStr">
@@ -49340,17 +49340,17 @@
       </c>
       <c r="BU92" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV92" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW92" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX92" t="inlineStr">
@@ -49398,7 +49398,7 @@
       </c>
       <c r="CG92" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH92" t="inlineStr">
@@ -49698,17 +49698,17 @@
       </c>
       <c r="BU93" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV93" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW93" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX93" t="inlineStr">
@@ -49756,7 +49756,7 @@
       </c>
       <c r="CG93" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH93" t="inlineStr">
@@ -50056,17 +50056,17 @@
       </c>
       <c r="BU94" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV94" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW94" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX94" t="inlineStr">
@@ -50114,7 +50114,7 @@
       </c>
       <c r="CG94" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH94" t="inlineStr">
@@ -50414,17 +50414,17 @@
       </c>
       <c r="BU95" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV95" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW95" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX95" t="inlineStr">
@@ -50472,7 +50472,7 @@
       </c>
       <c r="CG95" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH95" t="inlineStr">
@@ -50772,17 +50772,17 @@
       </c>
       <c r="BU96" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV96" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW96" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX96" t="inlineStr">
@@ -50830,7 +50830,7 @@
       </c>
       <c r="CG96" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH96" t="inlineStr">
@@ -51130,17 +51130,17 @@
       </c>
       <c r="BU97" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV97" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW97" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX97" t="inlineStr">
@@ -51188,7 +51188,7 @@
       </c>
       <c r="CG97" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH97" t="inlineStr">
@@ -51488,17 +51488,17 @@
       </c>
       <c r="BU98" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV98" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW98" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX98" t="inlineStr">
@@ -51546,7 +51546,7 @@
       </c>
       <c r="CG98" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH98" t="inlineStr">
@@ -51846,17 +51846,17 @@
       </c>
       <c r="BU99" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV99" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW99" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX99" t="inlineStr">
@@ -51904,7 +51904,7 @@
       </c>
       <c r="CG99" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH99" t="inlineStr">
@@ -52204,17 +52204,17 @@
       </c>
       <c r="BU100" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV100" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW100" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX100" t="inlineStr">
@@ -52262,7 +52262,7 @@
       </c>
       <c r="CG100" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH100" t="inlineStr">
@@ -52562,17 +52562,17 @@
       </c>
       <c r="BU101" t="inlineStr">
         <is>
-          <t>qualibact-v1.1</t>
+          <t>qualibact-v1.0</t>
         </is>
       </c>
       <c r="BV101" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="BW101" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="BX101" t="inlineStr">
@@ -52620,7 +52620,7 @@
       </c>
       <c r="CG101" t="inlineStr">
         <is>
-          <t>QualiBact Escherichia coli qualibact-v1.1</t>
+          <t>QualiBact Escherichia coli qualibact-v1.0</t>
         </is>
       </c>
       <c r="CH101" t="inlineStr">

</xml_diff>